<commit_message>
all scrapers should be done
</commit_message>
<xml_diff>
--- a/data/gas_flows.xlsx
+++ b/data/gas_flows.xlsx
@@ -959,34 +959,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>24</v>
+        <v>73.68000000000001</v>
       </c>
       <c r="C2" t="n">
-        <v>18</v>
+        <v>43.421</v>
       </c>
       <c r="D2" t="n">
-        <v>16</v>
+        <v>20.274</v>
       </c>
       <c r="E2" t="n">
-        <v>7</v>
-      </c>
-      <c r="F2" t="n">
-        <v>3.5</v>
+        <v>25.114</v>
       </c>
       <c r="G2" t="n">
-        <v>10</v>
+        <v>8.634</v>
       </c>
       <c r="H2" t="n">
-        <v>6</v>
+        <v>4.634</v>
       </c>
       <c r="I2" t="n">
-        <v>11</v>
+        <v>7.937</v>
       </c>
       <c r="J2" t="n">
-        <v>8</v>
+        <v>4.4</v>
       </c>
       <c r="K2" t="n">
-        <v>14.5</v>
+        <v>4.75</v>
       </c>
     </row>
     <row r="3">
@@ -996,34 +993,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>24.2</v>
+        <v>73.84999999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>18.1</v>
+        <v>43.696</v>
       </c>
       <c r="D3" t="n">
-        <v>16.2</v>
+        <v>18.185</v>
       </c>
       <c r="E3" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="F3" t="n">
-        <v>3.6</v>
+        <v>25.096</v>
       </c>
       <c r="G3" t="n">
-        <v>10.1</v>
+        <v>8.734</v>
       </c>
       <c r="H3" t="n">
-        <v>6.1</v>
+        <v>4.615</v>
       </c>
       <c r="I3" t="n">
-        <v>11.1</v>
+        <v>8.297000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>8.1</v>
+        <v>4.4</v>
       </c>
       <c r="K3" t="n">
-        <v>14.4</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="4">
@@ -1033,34 +1027,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>24.1</v>
+        <v>74.08</v>
       </c>
       <c r="C4" t="n">
-        <v>18</v>
+        <v>39.237</v>
       </c>
       <c r="D4" t="n">
-        <v>16</v>
+        <v>18.177</v>
       </c>
       <c r="E4" t="n">
-        <v>7</v>
-      </c>
-      <c r="F4" t="n">
-        <v>3.5</v>
+        <v>24.577</v>
       </c>
       <c r="G4" t="n">
-        <v>10</v>
+        <v>7.486</v>
       </c>
       <c r="H4" t="n">
-        <v>6</v>
+        <v>4.444</v>
       </c>
       <c r="I4" t="n">
-        <v>11</v>
+        <v>7.285</v>
       </c>
       <c r="J4" t="n">
-        <v>8</v>
+        <v>4.39</v>
       </c>
       <c r="K4" t="n">
-        <v>14.5</v>
+        <v>4.21</v>
       </c>
     </row>
     <row r="5">
@@ -1070,34 +1061,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>23.8</v>
+        <v>74.06999999999999</v>
       </c>
       <c r="C5" t="n">
-        <v>17.8</v>
+        <v>41.83</v>
       </c>
       <c r="D5" t="n">
-        <v>15.9</v>
+        <v>19.58</v>
       </c>
       <c r="E5" t="n">
-        <v>6.9</v>
-      </c>
-      <c r="F5" t="n">
-        <v>3.4</v>
+        <v>23.894</v>
       </c>
       <c r="G5" t="n">
-        <v>9.9</v>
+        <v>6.852</v>
       </c>
       <c r="H5" t="n">
-        <v>5.9</v>
+        <v>4.497</v>
       </c>
       <c r="I5" t="n">
-        <v>10.9</v>
+        <v>5.406</v>
       </c>
       <c r="J5" t="n">
-        <v>7.9</v>
+        <v>4.39</v>
       </c>
       <c r="K5" t="n">
-        <v>14.8</v>
+        <v>4.14</v>
       </c>
     </row>
     <row r="6">
@@ -1107,34 +1095,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>24</v>
+        <v>74.06</v>
       </c>
       <c r="C6" t="n">
-        <v>18.1</v>
+        <v>35.872</v>
       </c>
       <c r="D6" t="n">
-        <v>16.1</v>
+        <v>19.911</v>
       </c>
       <c r="E6" t="n">
-        <v>7</v>
-      </c>
-      <c r="F6" t="n">
-        <v>3.5</v>
+        <v>23.596</v>
       </c>
       <c r="G6" t="n">
-        <v>10</v>
+        <v>7.024</v>
       </c>
       <c r="H6" t="n">
-        <v>6</v>
+        <v>4.205</v>
       </c>
       <c r="I6" t="n">
-        <v>11.1</v>
+        <v>5.258</v>
       </c>
       <c r="J6" t="n">
-        <v>8.1</v>
+        <v>4.35</v>
       </c>
       <c r="K6" t="n">
-        <v>14.7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -1144,34 +1129,31 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>24.3</v>
+        <v>74.04000000000001</v>
       </c>
       <c r="C7" t="n">
-        <v>18.2</v>
+        <v>38.639</v>
       </c>
       <c r="D7" t="n">
-        <v>16.1</v>
+        <v>19.94</v>
       </c>
       <c r="E7" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="F7" t="n">
-        <v>3.6</v>
+        <v>24.675</v>
       </c>
       <c r="G7" t="n">
-        <v>10.1</v>
+        <v>7.819</v>
       </c>
       <c r="H7" t="n">
-        <v>6.1</v>
+        <v>4.031</v>
       </c>
       <c r="I7" t="n">
-        <v>11.2</v>
+        <v>5.445</v>
       </c>
       <c r="J7" t="n">
-        <v>8.1</v>
+        <v>4.25</v>
       </c>
       <c r="K7" t="n">
-        <v>14.6</v>
+        <v>4.27</v>
       </c>
     </row>
     <row r="8">
@@ -1181,34 +1163,31 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>74.15000000000001</v>
       </c>
       <c r="C8" t="n">
-        <v>18.1</v>
+        <v>27.482</v>
       </c>
       <c r="D8" t="n">
-        <v>16</v>
+        <v>20.392</v>
       </c>
       <c r="E8" t="n">
-        <v>7</v>
-      </c>
-      <c r="F8" t="n">
-        <v>3.5</v>
+        <v>25.054</v>
       </c>
       <c r="G8" t="n">
-        <v>10</v>
+        <v>7.419</v>
       </c>
       <c r="H8" t="n">
-        <v>6</v>
+        <v>3.616</v>
       </c>
       <c r="I8" t="n">
-        <v>11.1</v>
+        <v>5.831</v>
       </c>
       <c r="J8" t="n">
-        <v>8.1</v>
+        <v>4.06</v>
       </c>
       <c r="K8" t="n">
-        <v>15.2</v>
+        <v>4.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>